<commit_message>
Remove tab from markdown
</commit_message>
<xml_diff>
--- a/masterProjectList.xlsx
+++ b/masterProjectList.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ben Hess\Documents\GitHub\btmhess.github.io\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ben\Documents\GitHub\btmhess.github.io\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6CCF29D-8A4F-4B7E-8536-6926327DB759}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93E6A64A-54E1-478C-931D-FCC53B407B4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-83" yWindow="0" windowWidth="11686" windowHeight="13763" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="128">
   <si>
     <t>Goldwing tractive battery</t>
   </si>
@@ -417,6 +417,9 @@
   </si>
   <si>
     <t>complete_in_use</t>
+  </si>
+  <si>
+    <t>active</t>
   </si>
 </sst>
 </file>
@@ -787,18 +790,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:P53"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="44.28515625" customWidth="1"/>
-    <col min="2" max="2" width="18.28515625" customWidth="1"/>
-    <col min="3" max="3" width="21.28515625" customWidth="1"/>
-    <col min="4" max="4" width="12.7109375" customWidth="1"/>
-    <col min="5" max="5" width="9.7109375" customWidth="1"/>
-    <col min="8" max="8" width="9.42578125" customWidth="1"/>
-    <col min="10" max="10" width="9.5703125" customWidth="1"/>
-    <col min="12" max="12" width="12.28515625" customWidth="1"/>
-    <col min="13" max="14" width="10.28515625" customWidth="1"/>
-    <col min="15" max="15" width="11.42578125" customWidth="1"/>
+    <col min="1" max="1" width="44.265625" customWidth="1"/>
+    <col min="2" max="2" width="18.265625" customWidth="1"/>
+    <col min="3" max="3" width="21.265625" customWidth="1"/>
+    <col min="4" max="4" width="12.73046875" customWidth="1"/>
+    <col min="5" max="5" width="9.73046875" customWidth="1"/>
+    <col min="8" max="8" width="9.3984375" customWidth="1"/>
+    <col min="10" max="10" width="9.59765625" customWidth="1"/>
+    <col min="12" max="12" width="12.265625" customWidth="1"/>
+    <col min="13" max="14" width="10.265625" customWidth="1"/>
+    <col min="15" max="15" width="11.3984375" customWidth="1"/>
     <col min="16" max="16" width="12" customWidth="1"/>
   </cols>
   <sheetData>
@@ -945,6 +948,9 @@
       <c r="O3" t="s">
         <v>98</v>
       </c>
+      <c r="P3" t="s">
+        <v>98</v>
+      </c>
     </row>
     <row r="4" spans="1:16">
       <c r="A4" s="1" t="s">
@@ -967,6 +973,18 @@
       </c>
       <c r="G4">
         <v>75</v>
+      </c>
+      <c r="H4">
+        <v>100</v>
+      </c>
+      <c r="I4" t="s">
+        <v>127</v>
+      </c>
+      <c r="K4" t="s">
+        <v>98</v>
+      </c>
+      <c r="L4" t="s">
+        <v>98</v>
       </c>
       <c r="M4" t="s">
         <v>98</v>

</xml_diff>

<commit_message>
Publish 24s tractive battery
</commit_message>
<xml_diff>
--- a/masterProjectList.xlsx
+++ b/masterProjectList.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ben Hess\Documents\GitHub\btmhess.github.io\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ben\Documents\GitHub\btmhess.github.io\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B640D3D-C57C-4A63-98FA-AD61C03EE475}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24E91FC0-6AC6-4134-BA3F-1CCF26BAB3C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="130">
   <si>
     <t>Goldwing tractive battery</t>
   </si>
@@ -796,18 +796,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:P53"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="30.42578125" customWidth="1"/>
-    <col min="2" max="2" width="18.28515625" customWidth="1"/>
-    <col min="3" max="3" width="10.140625" customWidth="1"/>
-    <col min="4" max="4" width="7.7109375" customWidth="1"/>
-    <col min="5" max="5" width="9.7109375" customWidth="1"/>
-    <col min="8" max="8" width="9.42578125" customWidth="1"/>
-    <col min="10" max="10" width="9.5703125" customWidth="1"/>
-    <col min="12" max="12" width="12.28515625" customWidth="1"/>
-    <col min="13" max="14" width="10.28515625" customWidth="1"/>
-    <col min="15" max="15" width="11.42578125" customWidth="1"/>
+    <col min="1" max="1" width="30.3984375" customWidth="1"/>
+    <col min="2" max="2" width="18.265625" customWidth="1"/>
+    <col min="3" max="3" width="10.1328125" customWidth="1"/>
+    <col min="4" max="4" width="7.73046875" customWidth="1"/>
+    <col min="5" max="5" width="9.73046875" customWidth="1"/>
+    <col min="8" max="8" width="9.3984375" customWidth="1"/>
+    <col min="10" max="10" width="9.59765625" customWidth="1"/>
+    <col min="12" max="12" width="12.265625" customWidth="1"/>
+    <col min="13" max="14" width="10.265625" customWidth="1"/>
+    <col min="15" max="15" width="11.3984375" customWidth="1"/>
     <col min="16" max="16" width="12" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1150,7 +1150,28 @@
       <c r="G8">
         <v>16</v>
       </c>
+      <c r="H8">
+        <v>1143</v>
+      </c>
+      <c r="I8" t="s">
+        <v>128</v>
+      </c>
+      <c r="J8" t="s">
+        <v>41</v>
+      </c>
+      <c r="K8" t="s">
+        <v>97</v>
+      </c>
+      <c r="L8" t="s">
+        <v>97</v>
+      </c>
       <c r="M8" t="s">
+        <v>97</v>
+      </c>
+      <c r="O8" t="s">
+        <v>97</v>
+      </c>
+      <c r="P8" t="s">
         <v>97</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish INP and motor bycicle
</commit_message>
<xml_diff>
--- a/masterProjectList.xlsx
+++ b/masterProjectList.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ben\Documents\GitHub\btmhess.github.io\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24E91FC0-6AC6-4134-BA3F-1CCF26BAB3C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{451AA615-3108-4DEA-ADE2-5490D5B8A2F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="131">
   <si>
     <t>Goldwing tractive battery</t>
   </si>
@@ -426,6 +426,9 @@
   </si>
   <si>
     <t>Quadwood Go-Kart</t>
+  </si>
+  <si>
+    <t>complete_abandoned</t>
   </si>
 </sst>
 </file>
@@ -1197,6 +1200,21 @@
       <c r="G9">
         <v>70</v>
       </c>
+      <c r="H9">
+        <v>1000</v>
+      </c>
+      <c r="I9" t="s">
+        <v>130</v>
+      </c>
+      <c r="J9" t="s">
+        <v>41</v>
+      </c>
+      <c r="K9" t="s">
+        <v>97</v>
+      </c>
+      <c r="L9" t="s">
+        <v>97</v>
+      </c>
       <c r="M9" t="s">
         <v>97</v>
       </c>
@@ -1223,7 +1241,22 @@
       <c r="G10">
         <v>16</v>
       </c>
+      <c r="H10">
+        <v>7500</v>
+      </c>
+      <c r="I10" t="s">
+        <v>125</v>
+      </c>
+      <c r="K10" t="s">
+        <v>97</v>
+      </c>
+      <c r="L10" t="s">
+        <v>97</v>
+      </c>
       <c r="M10" t="s">
+        <v>97</v>
+      </c>
+      <c r="O10" t="s">
         <v>97</v>
       </c>
     </row>

</xml_diff>